<commit_message>
added tri6, quad8, and quad9 elements to mesh generation. updated seep.py to work with tri6 elements.
</commit_message>
<xml_diff>
--- a/inputs/slope/input_template_lface5.xlsx
+++ b/inputs/slope/input_template_lface5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jones/CursorProjects/xslope/inputs/slope/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2616612-3379-384D-B01E-B8195039E7BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{513A1566-8232-BC4B-AB3F-541A784F41AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3060" yWindow="880" windowWidth="29340" windowHeight="17300" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="3060" yWindow="880" windowWidth="29340" windowHeight="17300" activeTab="9" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -5669,7 +5669,7 @@
         <v>111</v>
       </c>
       <c r="C3" s="31">
-        <v>302</v>
+        <v>80</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>111</v>
@@ -6380,16 +6380,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="G22:H22"/>
     <mergeCell ref="J22:K22"/>
     <mergeCell ref="M22:N22"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>